<commit_message>
Add patient appointment test cases
</commit_message>
<xml_diff>
--- a/Test Cases.xlsx
+++ b/Test Cases.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Garry Albis\Downloads\Greg\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Garry Albis\Downloads\Greg\Test Cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ED97B29-F38A-49D3-9300-D4D84A68F69E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8628734D-8AA2-4649-A487-322BA09836EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{AD39C554-7331-4D09-A6DF-3146592A8CEE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{AD39C554-7331-4D09-A6DF-3146592A8CEE}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Scenario" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="242">
   <si>
     <t>TS-001</t>
   </si>
@@ -268,9 +268,6 @@
     <t>User only see dots in password</t>
   </si>
   <si>
-    <t>User is prevented from logging in with invalid credentials</t>
-  </si>
-  <si>
     <t>User can log in using Google authentication</t>
   </si>
   <si>
@@ -334,15 +331,6 @@
     <t>Password is securely masked during login</t>
   </si>
   <si>
-    <t>Admi can login and access the admin dashboard</t>
-  </si>
-  <si>
-    <t>Dentist can login and access the dentist dashboard</t>
-  </si>
-  <si>
-    <t>Staff can login and access the staff dashboard</t>
-  </si>
-  <si>
     <t>TS-007</t>
   </si>
   <si>
@@ -376,9 +364,6 @@
     <t>Users changed their password and redirected to the login page</t>
   </si>
   <si>
-    <t>User successfully change their password and directed to the login page</t>
-  </si>
-  <si>
     <t>Forgot password with unregistered account</t>
   </si>
   <si>
@@ -389,9 +374,6 @@
   </si>
   <si>
     <t>Users didn’t receive OTP and "Cant find a user with that email address" appear</t>
-  </si>
-  <si>
-    <t>Users didn’t reiceive OTP code and error "Cant find that email address" appeared</t>
   </si>
   <si>
     <t>Forgot Password with empty email address</t>
@@ -461,9 +443,6 @@
 Confirm Password: 1234567</t>
   </si>
   <si>
-    <t>User password didn’t change and the password must be 8 character or more appear</t>
-  </si>
-  <si>
     <t>Verify new/Reset password with new password and confirm password unmatch</t>
   </si>
   <si>
@@ -478,9 +457,6 @@
   </si>
   <si>
     <t>Verify new/reset password with expired link</t>
-  </si>
-  <si>
-    <t>The link receive link is expired</t>
   </si>
   <si>
     <t>1. Go to login page 
@@ -647,6 +623,378 @@
   </si>
   <si>
     <t>Test Scenario ID</t>
+  </si>
+  <si>
+    <t>TS-009</t>
+  </si>
+  <si>
+    <t>TS-010</t>
+  </si>
+  <si>
+    <t>TS-011</t>
+  </si>
+  <si>
+    <t>TC-023</t>
+  </si>
+  <si>
+    <t>TS-012</t>
+  </si>
+  <si>
+    <t>Patient make an appointment for themself</t>
+  </si>
+  <si>
+    <t>First Name: Juan
+Last Name: Dela Cruz
+Middle Name: Luna
+Birth Date: 25/10/2003
+Contact Number: 09123123123
+Email Address: Patient@gmail.com</t>
+  </si>
+  <si>
+    <t>1. Go to the website
+2. Click book appointment
+3. Click "For Myself"
+4. Enter First Name
+5. Enter Last Name
+6. Enter Middle Name
+7. Enter Birth Date
+8. Enter Contact Number
+9. Enter Email Address
+10. Select Services
+11. Pick Dates of your appointment
+12. Select Time
+13. Complete reCaptcha
+14. Check Agreement
+15. Click Confirm Appointment button</t>
+  </si>
+  <si>
+    <t>1. Go to the website
+2. Click book appointment
+3. Click "For Myself"
+4. Enter First Name
+5. Enter Last Name
+6. Enter Middle Name
+7. Enter Birth Date
+8. Enter Contact Number
+9. Enter Email Address
+10. Select Services
+11. Pick Dates of your appointment
+12. Select Time
+13. Complete reCaptcha
+14. Check Agreement
+15. Click Confirm Appointment button
+16. Go to your email
+17. Copy the OTP
+18. Go back to the website
+19. Paste the OTP
+20. Click Verify &amp; Book button</t>
+  </si>
+  <si>
+    <t>Patient successfully book an appointment and "Book Appointment Displayed" and receive email notification</t>
+  </si>
+  <si>
+    <t>Patient can book appointment for their relatives using his/her email address</t>
+  </si>
+  <si>
+    <t>Patient book appointment for someone else</t>
+  </si>
+  <si>
+    <t>Contact First Name: Emu
+Contact Last Name: Otori
+Contact Middle Name: Park
+Contact Number: 09982231277
+Email Address: Mother@gmail.com
+Patient First Name: Nene
+Patient Last Name: Otori
+Patient Middle Name: Park
+Patient Birth Date: 20/7/2010
+Relationship to Patient: Mother</t>
+  </si>
+  <si>
+    <t>1. Go to the website
+2. Click book appointment
+3. Click "For Someone Else"
+4. Enter Contact First Name
+5. Enter Contact Last Name
+6. Enter Contact Middle Name
+7. Enter Contact Number
+8. Enter Contact Email Address
+9. Enter Patient First Name
+10. Enter Patient Last Name
+11. Enter Patient Middle Name
+12. Enter Patient Birth Date
+13. Enter Relationship to Patient
+14. Select Services
+15. Pick Dates of your appointment
+16. Select Time
+17. Complete reCaptcha
+18. Check Agreement
+19. Click Confirm Appointment button
+20. Go to your email
+21. Copy the OTP
+22. Go back to the website
+23. Paste the OTP
+24. Click Verify &amp; Book button</t>
+  </si>
+  <si>
+    <t>TC-024</t>
+  </si>
+  <si>
+    <t>Patient have an existing appointment</t>
+  </si>
+  <si>
+    <t>Patient can't proceed to book appointment with existing appointment request</t>
+  </si>
+  <si>
+    <t>Patient didn’t proceed to the book appointment and "Already have pending or upcoming appointment request" displayed</t>
+  </si>
+  <si>
+    <t>TC-025</t>
+  </si>
+  <si>
+    <t>Patient can't proceed to book appointment with incomplete required information</t>
+  </si>
+  <si>
+    <t>First Name: Juan
+Last Name:
+Middle Name: Luna
+Birth Date: 25/10/2003
+Contact Number: 09123123123
+Email Address: Patient@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Go to the website
+2. Click book appointment
+3. Click "For Myself"
+4. Enter First Name
+5. Enter Last Name
+6. Enter Middle Name
+7. Enter Birth Date
+8. Enter Contact Number
+9. Enter Email Address
+10. Select Services
+11. Pick Dates of your appointment
+12. Select Time
+13. Complete reCaptcha
+14. Check Agreement
+15. Click Confirm Appointment button
+</t>
+  </si>
+  <si>
+    <t>Patient didn’t proceed to the book appointment and required missing fields is highlighted</t>
+  </si>
+  <si>
+    <t>Patient didn’t proceed to the book appointment and required missing fields are highlighted</t>
+  </si>
+  <si>
+    <t>TC-026</t>
+  </si>
+  <si>
+    <t>Verify that OTP is expired after 3 minutes</t>
+  </si>
+  <si>
+    <t>TC-027</t>
+  </si>
+  <si>
+    <t>Patient receive new OTP code</t>
+  </si>
+  <si>
+    <t>1. Go to the website
+2. Click book appointment
+3. Click "For Myself"
+4. Enter First Name
+5. Enter Last Name
+6. Enter Middle Name
+7. Enter Birth Date
+8. Enter Contact Number
+9. Enter Email Address
+10. Select Services
+11. Pick Dates of your appointment
+12. Select Time
+13. Complete reCaptcha
+14. Check Agreement
+15. Click Confirm Appointment button
+16. Go to your email
+17. Verify it send OTP
+18. Go back to the website
+19. Click Resent OTP
+20. Verify receive new OTP</t>
+  </si>
+  <si>
+    <t>Patient received new OTP code</t>
+  </si>
+  <si>
+    <t>"Expired OTP" displayed</t>
+  </si>
+  <si>
+    <t>Patient already receive 3 OTP</t>
+  </si>
+  <si>
+    <t>click resend OTP 3 times</t>
+  </si>
+  <si>
+    <t>Verify that Patient didn’t receive success appointment without OTP code</t>
+  </si>
+  <si>
+    <t>Patient didn’t enter OTP code</t>
+  </si>
+  <si>
+    <t>No OTP code</t>
+  </si>
+  <si>
+    <t>1. Go to the website
+2. Click book appointment
+3. Click "For Myself"
+4. Enter First Name
+5. Enter Last Name
+6. Enter Middle Name
+7. Enter Birth Date
+8. Enter Contact Number
+9. Enter Email Address
+10. Select Services
+11. Pick Dates of your appointment
+12. Select Time
+13. Complete reCaptcha
+14. Check Agreement
+15. Click Confirm Appointment button
+16. Click Verify &amp; Book button</t>
+  </si>
+  <si>
+    <t>"Enter OTP" displayed and Highlighted</t>
+  </si>
+  <si>
+    <t>TS-013</t>
+  </si>
+  <si>
+    <t>TC-029</t>
+  </si>
+  <si>
+    <t>TC-028</t>
+  </si>
+  <si>
+    <t>TC-030</t>
+  </si>
+  <si>
+    <t>Patients can book an appointment for themselves</t>
+  </si>
+  <si>
+    <t>patient can book an appointment for someone else</t>
+  </si>
+  <si>
+    <t>Verify that a patient cannot book another appointment when an existing appointment is pending or upcoming</t>
+  </si>
+  <si>
+    <t>Verify that a patient cannot book an appointment with incomplete required information</t>
+  </si>
+  <si>
+    <t>Verify that the OTP function works as expected</t>
+  </si>
+  <si>
+    <t>1. Go to the website
+2. Click book appointment
+3. Click "For Myself"
+4. Enter First Name
+5. Enter Last Name
+6. Enter Middle Name
+7. Enter Birth Date
+8. Enter Contact Number
+9. Enter Email Address
+10. Select Services
+11. Pick Dates of your appointment
+12. Select Time
+13. Complete reCaptcha
+14. Check Agreement
+15. Click Confirm Appointment button
+16. Go to your email
+17. Copy the OTP
+18. Go back to the website
+19. Wait for 3 minutes
+20. Paste the OTP
+21. Click Verify &amp; Book button</t>
+  </si>
+  <si>
+    <t>Verify it send OTP</t>
+  </si>
+  <si>
+    <t>1. Go to the website
+2. Click book appointment
+3. Click "For Myself"
+4. Enter First Name
+5. Enter Last Name
+6. Enter Middle Name
+7. Enter Birth Date
+8. Enter Contact Number
+9. Enter Email Address
+10. Select Services
+11. Pick Dates of your appointment
+12. Select Time
+13. Complete reCaptcha
+14. Check Agreement
+15. Click Confirm Appointment button
+16. Go to your email
+17. Verify it send OTP
+18. Go back to the website
+19. Click Resend OTP
+20. Wait for 1 minute to click Resend OTP
+21. Click Resend OTP again
+22. Do it until the OTP resend attempt counter reaches 3/3</t>
+  </si>
+  <si>
+    <t>"OTP Expired" is displayed and the appointment is not booked</t>
+  </si>
+  <si>
+    <t>The appointment is not booked and an "Enter OTP" validation message is displayed</t>
+  </si>
+  <si>
+    <t>Verify OTP can resend 3 times</t>
+  </si>
+  <si>
+    <t>The Patient doesn’t have upcoming appointment</t>
+  </si>
+  <si>
+    <t>"Appointment Booked" is displayed and the Patient receives an email notification containing the appointment details</t>
+  </si>
+  <si>
+    <t>Verify that an OTP is sent to the Patient's email address</t>
+  </si>
+  <si>
+    <t>After the maximum number of resend attempts is reached, the Resend OTP option is disabled and the Patient must wait 10 minutes before requesting another OTP</t>
+  </si>
+  <si>
+    <t>Resend OTP button is disabled and Patient need to wait 10 minutes</t>
+  </si>
+  <si>
+    <t>Users are prevented from logging in with invalid credentials</t>
+  </si>
+  <si>
+    <t>Admin can log in and access the admin dashboard</t>
+  </si>
+  <si>
+    <t>Dentist can log in and access the dentist dashboard</t>
+  </si>
+  <si>
+    <t>Staff can log in and access the staff dashboard</t>
+  </si>
+  <si>
+    <t>Patient have incomplete required information</t>
+  </si>
+  <si>
+    <t>User successfully changed their password and directed to the login page</t>
+  </si>
+  <si>
+    <t>The link received link is expired</t>
+  </si>
+  <si>
+    <t>Users didn’t receive OTP code and error "Cant find that email address" appeared</t>
+  </si>
+  <si>
+    <t>User password didn’t change and the password must be 8 characters or more appear</t>
+  </si>
+  <si>
+    <t>A valid OTP has been received and is ready to be used.</t>
+  </si>
+  <si>
+    <t>OTP Expiration: 3 minutes</t>
   </si>
 </sst>
 </file>
@@ -1044,7 +1392,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08C3A4CF-1E2B-49AB-82C3-D369404FBDB7}">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.5703125" style="1" bestFit="1" customWidth="1"/>
@@ -1061,7 +1409,7 @@
     <row r="3" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
       <c r="A3" s="3"/>
       <c r="B3" s="10" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="C3" s="10" t="s">
         <v>1</v>
@@ -1073,7 +1421,7 @@
         <v>0</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>90</v>
+        <v>232</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1082,7 +1430,7 @@
         <v>2</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>91</v>
+        <v>233</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1091,7 +1439,7 @@
         <v>3</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>92</v>
+        <v>234</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -1100,7 +1448,7 @@
         <v>4</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>68</v>
+        <v>231</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -1109,7 +1457,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -1118,31 +1466,75 @@
         <v>39</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
       <c r="B10" s="6" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="3"/>
       <c r="B11" s="6" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
+      <c r="B12" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B13" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="B14" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="B15" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B16" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1151,14 +1543,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5906D774-767F-4BAB-8C3F-52A1329D327D}">
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="24.140625" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="33.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="28.85546875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="31.5703125" style="2" customWidth="1"/>
     <col min="6" max="6" width="38.42578125" style="2" customWidth="1"/>
     <col min="7" max="7" width="23.28515625" style="4" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="19.85546875" style="4" bestFit="1" customWidth="1"/>
@@ -1199,7 +1591,7 @@
     </row>
     <row r="4" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>22</v>
@@ -1214,7 +1606,7 @@
         <v>35</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>17</v>
@@ -1225,7 +1617,7 @@
     </row>
     <row r="5" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>21</v>
@@ -1240,7 +1632,7 @@
         <v>36</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H5" s="4" t="s">
         <v>24</v>
@@ -1251,7 +1643,7 @@
     </row>
     <row r="6" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>25</v>
@@ -1266,7 +1658,7 @@
         <v>36</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>28</v>
@@ -1277,10 +1669,10 @@
     </row>
     <row r="7" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>30</v>
@@ -1292,7 +1684,7 @@
         <v>37</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>31</v>
@@ -1303,7 +1695,7 @@
     </row>
     <row r="8" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>32</v>
@@ -1318,7 +1710,7 @@
         <v>44</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H8" s="4" t="s">
         <v>38</v>
@@ -1329,7 +1721,7 @@
     </row>
     <row r="9" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>41</v>
@@ -1344,7 +1736,7 @@
         <v>43</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H9" s="4" t="s">
         <v>38</v>
@@ -1355,7 +1747,7 @@
     </row>
     <row r="10" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>45</v>
@@ -1370,7 +1762,7 @@
         <v>48</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>38</v>
@@ -1381,7 +1773,7 @@
     </row>
     <row r="11" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="B11" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>49</v>
@@ -1396,7 +1788,7 @@
         <v>52</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>53</v>
@@ -1407,7 +1799,7 @@
     </row>
     <row r="12" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="B12" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>61</v>
@@ -1422,7 +1814,7 @@
         <v>62</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H12" s="4" t="s">
         <v>57</v>
@@ -1433,7 +1825,7 @@
     </row>
     <row r="13" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="B13" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>54</v>
@@ -1448,7 +1840,7 @@
         <v>63</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H13" s="4" t="s">
         <v>58</v>
@@ -1459,10 +1851,10 @@
     </row>
     <row r="14" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>64</v>
@@ -1474,7 +1866,7 @@
         <v>66</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H14" s="4" t="s">
         <v>67</v>
@@ -1483,53 +1875,53 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="165" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" ht="150" x14ac:dyDescent="0.25">
       <c r="B15" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="D15" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="G15" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="D15" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="E15" s="4" t="s">
+      <c r="H15" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="B16" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="F15" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="G15" s="4" t="s">
+      <c r="D16" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="G16" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="H15" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="I15" s="4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="90" x14ac:dyDescent="0.25">
-      <c r="B16" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="G16" s="4" t="s">
-        <v>108</v>
-      </c>
       <c r="H16" s="4" t="s">
-        <v>109</v>
+        <v>238</v>
       </c>
       <c r="I16" s="4" t="s">
         <v>18</v>
@@ -1537,25 +1929,25 @@
     </row>
     <row r="17" spans="2:9" ht="60" x14ac:dyDescent="0.25">
       <c r="B17" s="2" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="I17" s="4" t="s">
         <v>18</v>
@@ -1563,209 +1955,417 @@
     </row>
     <row r="18" spans="2:9" ht="60" x14ac:dyDescent="0.25">
       <c r="B18" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="D18" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="E18" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="I18" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="19" spans="2:9" ht="150" x14ac:dyDescent="0.25">
+      <c r="B19" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="D19" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="E19" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="F19" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="I19" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="2:9" ht="150" x14ac:dyDescent="0.25">
+      <c r="B20" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C20" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="F18" s="4" t="s">
+      <c r="D20" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="G18" s="4" t="s">
+      <c r="E20" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21" spans="2:9" ht="105" x14ac:dyDescent="0.25">
+      <c r="B21" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="22" spans="2:9" ht="150" x14ac:dyDescent="0.25">
+      <c r="B22" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="I22" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="23" spans="2:9" ht="105" x14ac:dyDescent="0.25">
+      <c r="B23" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="C23" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="H18" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="I18" s="4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="19" spans="2:9" ht="165" x14ac:dyDescent="0.25">
-      <c r="B19" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="F19" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="G19" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="H19" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="I19" s="4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="20" spans="2:9" ht="165" x14ac:dyDescent="0.25">
-      <c r="B20" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="F20" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="G20" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="H20" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="I20" s="4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="21" spans="2:9" ht="135" x14ac:dyDescent="0.25">
-      <c r="B21" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="F21" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="G21" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="H21" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="I21" s="4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="22" spans="2:9" ht="165" x14ac:dyDescent="0.25">
-      <c r="B22" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="G22" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="H22" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="I22" s="4" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="23" spans="2:9" ht="120" x14ac:dyDescent="0.25">
-      <c r="B23" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>166</v>
-      </c>
       <c r="D23" s="4" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>27</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="I23" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="2:9" ht="120" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:9" ht="105" x14ac:dyDescent="0.25">
       <c r="B24" s="2" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>23</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="G24" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="H24" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="H24" s="4" t="s">
-        <v>177</v>
-      </c>
       <c r="I24" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="2:9" ht="120" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:9" ht="90" x14ac:dyDescent="0.25">
       <c r="B25" s="2" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="E25" s="4" t="s">
         <v>16</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="G25" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="26" spans="2:9" ht="300" x14ac:dyDescent="0.25">
+      <c r="B26" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="H25" s="4" t="s">
+      <c r="C26" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="I25" s="2" t="s">
+      <c r="D26" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="27" spans="2:9" ht="360" x14ac:dyDescent="0.25">
+      <c r="B27" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="28" spans="2:9" ht="240" x14ac:dyDescent="0.25">
+      <c r="B28" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="H28" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="29" spans="2:9" ht="225" x14ac:dyDescent="0.25">
+      <c r="B29" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="H29" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="30" spans="2:9" ht="315" x14ac:dyDescent="0.25">
+      <c r="B30" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="H30" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="31" spans="2:9" ht="300" x14ac:dyDescent="0.25">
+      <c r="B31" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="H31" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="32" spans="2:9" ht="345" x14ac:dyDescent="0.25">
+      <c r="B32" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="H32" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="33" spans="2:9" ht="240" x14ac:dyDescent="0.25">
+      <c r="B33" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="H33" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="I33" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1793,18 +2393,18 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B3" s="7" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>8</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="E3" s="8" t="s">
         <v>12</v>
@@ -1813,10 +2413,10 @@
         <v>13</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="I3" s="7" t="s">
         <v>14</v>
@@ -1824,28 +2424,28 @@
     </row>
     <row r="4" spans="1:9" ht="150" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>154</v>
-      </c>
       <c r="D4" s="4" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>